<commit_message>
Added line_number to long_df
used for multiple labels in the same episode id
</commit_message>
<xml_diff>
--- a/llacie/vocabs/cleaned_antibiotics.xlsx
+++ b/llacie/vocabs/cleaned_antibiotics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anish/Code/Pak Lab/llacie/llacie/database/use_this_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anish/Code/Pak Lab/llacie/llacie/vocabs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{741D32F5-55F7-9543-BCEA-73E5DDE780E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129D0A10-7046-784D-88ED-063AAE900ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Brand Names" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="321">
   <si>
     <t>Drug Name</t>
   </si>
@@ -34,9 +34,6 @@
     <t xml:space="preserve"> ERROR</t>
   </si>
   <si>
-    <t xml:space="preserve">trimethoprim/sulfamethoxazole </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Bactrim, Cotrim, Septra, others</t>
   </si>
   <si>
@@ -46,9 +43,6 @@
     <t xml:space="preserve"> Amikin, Amiglyde-V, Arikayce, others</t>
   </si>
   <si>
-    <t xml:space="preserve">amoxicillin/clavulanate </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Augmentin, Clavulin, Amoclan, others[1]</t>
   </si>
   <si>
@@ -58,9 +52,6 @@
     <t xml:space="preserve"> Principen, others[3]</t>
   </si>
   <si>
-    <t xml:space="preserve">ampicillin/sulbactam </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Unasyn</t>
   </si>
   <si>
@@ -166,9 +157,6 @@
     <t xml:space="preserve"> Pipracil</t>
   </si>
   <si>
-    <t xml:space="preserve">piperacillin/tazobactam </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Tazocin, Zosyn, others[1]</t>
   </si>
   <si>
@@ -235,9 +223,6 @@
     <t xml:space="preserve"> Eryc, Erythrocin, others[1]</t>
   </si>
   <si>
-    <t xml:space="preserve">quinupristin/dalfopristin </t>
-  </si>
-  <si>
     <t xml:space="preserve">voriconazole </t>
   </si>
   <si>
@@ -256,9 +241,6 @@
     <t xml:space="preserve"> Cubicin, Cubicin RF, Dapzura RT</t>
   </si>
   <si>
-    <t xml:space="preserve">beta/lactamase </t>
-  </si>
-  <si>
     <t xml:space="preserve">streptomycin </t>
   </si>
   <si>
@@ -310,9 +292,6 @@
     <t xml:space="preserve"> Ancobon, Ancotil, others</t>
   </si>
   <si>
-    <t xml:space="preserve">amphotericin/B </t>
-  </si>
-  <si>
     <t xml:space="preserve">anidulafungin </t>
   </si>
   <si>
@@ -334,15 +313,9 @@
     <t xml:space="preserve">eravacycline </t>
   </si>
   <si>
-    <t xml:space="preserve">meropenem/vaborbactam </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Vabomere, Vaborem, others</t>
   </si>
   <si>
-    <t xml:space="preserve">ceftazidime/avibactam </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Avycaz, Zavicefta, others[1]</t>
   </si>
   <si>
@@ -358,9 +331,6 @@
     <t xml:space="preserve"> Proloprim, Monotrim, Triprim, others</t>
   </si>
   <si>
-    <t xml:space="preserve">ceftolozane/tazobactam </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Zerbaxa</t>
   </si>
   <si>
@@ -391,18 +361,9 @@
     <t xml:space="preserve">ticarcillin </t>
   </si>
   <si>
-    <t xml:space="preserve">azithromycin </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Sumamed, Hemomicin, Zithromax, others[1]</t>
   </si>
   <si>
-    <t xml:space="preserve">penicillin/binding/protein/2a </t>
-  </si>
-  <si>
-    <t xml:space="preserve">extended/spectrum/beta/lactamase </t>
-  </si>
-  <si>
     <t xml:space="preserve">sulfamethoxazole </t>
   </si>
   <si>
@@ -418,15 +379,6 @@
     <t xml:space="preserve"> Cresemba</t>
   </si>
   <si>
-    <t xml:space="preserve">carbapenemase/other </t>
-  </si>
-  <si>
-    <t xml:space="preserve">imipenem/relebactam </t>
-  </si>
-  <si>
-    <t xml:space="preserve">inducible/clindamycin/resistance </t>
-  </si>
-  <si>
     <t xml:space="preserve">pyrazinamide </t>
   </si>
   <si>
@@ -466,21 +418,6 @@
     <t xml:space="preserve"> Capastat</t>
   </si>
   <si>
-    <t xml:space="preserve">carbapenemase/ndm </t>
-  </si>
-  <si>
-    <t xml:space="preserve">carbapenemase/vim </t>
-  </si>
-  <si>
-    <t xml:space="preserve">carbapenemase/imp </t>
-  </si>
-  <si>
-    <t xml:space="preserve">carbapenemase/kpc </t>
-  </si>
-  <si>
-    <t xml:space="preserve">carbapenemase/oxa </t>
-  </si>
-  <si>
     <t xml:space="preserve">terbinafine </t>
   </si>
   <si>
@@ -511,9 +448,6 @@
     <t xml:space="preserve"> Trobicin</t>
   </si>
   <si>
-    <t xml:space="preserve">ethambutol/rifampin </t>
-  </si>
-  <si>
     <t xml:space="preserve">telavancin </t>
   </si>
   <si>
@@ -562,24 +496,12 @@
     <t xml:space="preserve"> Baxdela, others</t>
   </si>
   <si>
-    <t xml:space="preserve">sulbactam/durlobactam </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Xacduro</t>
   </si>
   <si>
-    <t xml:space="preserve">aztreonam/avibactam </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Emblaveo</t>
   </si>
   <si>
-    <t xml:space="preserve">ceftazidime/clavulanate </t>
-  </si>
-  <si>
-    <t xml:space="preserve">cefotaxime/clavulanate </t>
-  </si>
-  <si>
     <t xml:space="preserve">miconazole </t>
   </si>
   <si>
@@ -604,12 +526,6 @@
     <t xml:space="preserve"> Nizoral, others</t>
   </si>
   <si>
-    <t xml:space="preserve">polymyxin/B </t>
-  </si>
-  <si>
-    <t xml:space="preserve">meropenem/imipenem </t>
-  </si>
-  <si>
     <t xml:space="preserve">nystatin </t>
   </si>
   <si>
@@ -634,9 +550,6 @@
     <t xml:space="preserve"> Lotrimin, others</t>
   </si>
   <si>
-    <t xml:space="preserve">nalidixic/acid </t>
-  </si>
-  <si>
     <t xml:space="preserve">ceftizoxime </t>
   </si>
   <si>
@@ -646,9 +559,6 @@
     <t xml:space="preserve">cefoperazone </t>
   </si>
   <si>
-    <t xml:space="preserve">fusidic/acid </t>
-  </si>
-  <si>
     <t xml:space="preserve">azlocillin </t>
   </si>
   <si>
@@ -748,9 +658,6 @@
     <t xml:space="preserve"> Netromycin</t>
   </si>
   <si>
-    <t xml:space="preserve">p/aminosalicylic/acid </t>
-  </si>
-  <si>
     <t xml:space="preserve">sparfloxacin </t>
   </si>
   <si>
@@ -775,9 +682,6 @@
     <t xml:space="preserve"> Conteben</t>
   </si>
   <si>
-    <t xml:space="preserve">ticarcillin/clavulanate </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Timentin</t>
   </si>
   <si>
@@ -904,9 +808,6 @@
     <t xml:space="preserve">paromomycin </t>
   </si>
   <si>
-    <t xml:space="preserve"> Catenulin, Aminosidine, Humatin, others[1]</t>
-  </si>
-  <si>
     <t xml:space="preserve">retampulin </t>
   </si>
   <si>
@@ -949,9 +850,6 @@
     <t>Recarbrio</t>
   </si>
   <si>
-    <t>Not sure about this: Site uses this https://en.wikipedia.org/wiki/Imipenem/cilastatin/relebactam</t>
-  </si>
-  <si>
     <t>Fucidin, Foban</t>
   </si>
   <si>
@@ -965,13 +863,133 @@
   </si>
   <si>
     <t>Mandol</t>
+  </si>
+  <si>
+    <t>Gris-peg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trimethoprim_sulfamethoxazole </t>
+  </si>
+  <si>
+    <t xml:space="preserve">amoxicillin_clavulanate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ampicillin_sulbactam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">piperacillin_tazobactam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">quinupristin_dalfopristin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">beta_lactamase </t>
+  </si>
+  <si>
+    <t xml:space="preserve">amphotericin_B </t>
+  </si>
+  <si>
+    <t xml:space="preserve">meropenem_vaborbactam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceftazidime_avibactam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceftolozane_tazobactam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">penicillin_binding_protein_2a </t>
+  </si>
+  <si>
+    <t xml:space="preserve">extended_spectrum_beta_lactamase </t>
+  </si>
+  <si>
+    <t xml:space="preserve">carbapenemase_other </t>
+  </si>
+  <si>
+    <t xml:space="preserve">imipenem_relebactam </t>
+  </si>
+  <si>
+    <t>Not sure about this: Site uses this https:__en.wikipedia.org_wiki_Imipenem_cilastatin_relebactam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inducible_clindamycin_resistance </t>
+  </si>
+  <si>
+    <t xml:space="preserve">carbapenemase_ndm </t>
+  </si>
+  <si>
+    <t xml:space="preserve">carbapenemase_vim </t>
+  </si>
+  <si>
+    <t xml:space="preserve">carbapenemase_imp </t>
+  </si>
+  <si>
+    <t xml:space="preserve">carbapenemase_kpc </t>
+  </si>
+  <si>
+    <t xml:space="preserve">carbapenemase_oxa </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethambutol_rifampin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">sulbactam_durlobactam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">aztreonam_avibactam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceftazidime_clavulanate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cefotaxime_clavulanate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">polymyxin_B </t>
+  </si>
+  <si>
+    <t xml:space="preserve">meropenem_imipenem </t>
+  </si>
+  <si>
+    <t xml:space="preserve">nalidixic_acid </t>
+  </si>
+  <si>
+    <t xml:space="preserve">fusidic_acid </t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_aminosalicylic_acid </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ticarcillin_clavulanate </t>
+  </si>
+  <si>
+    <t>azithromycin</t>
+  </si>
+  <si>
+    <t>Added my own from here</t>
+  </si>
+  <si>
+    <t>sulfadiazine</t>
+  </si>
+  <si>
+    <t>pyrimethamine</t>
+  </si>
+  <si>
+    <t>Daraprim</t>
+  </si>
+  <si>
+    <t>benzathine penicillin</t>
+  </si>
+  <si>
+    <t>Bicillin L-A, Permapen,benzyl, penicillin G benzathine, benzylpenicillin benzathine</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -979,8 +997,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1005,6 +1029,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1018,11 +1048,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1346,7 +1377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.5" customWidth="1"/>
@@ -1377,10 +1408,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C3" t="s">
         <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1388,10 +1419,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
         <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1399,10 +1430,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>283</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1410,10 +1441,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1421,10 +1452,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>284</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -1432,10 +1463,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -1443,10 +1474,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -1454,10 +1485,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -1465,10 +1496,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -1476,10 +1507,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -1487,10 +1518,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -1498,10 +1529,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -1509,10 +1540,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -1520,10 +1551,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C16" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -1531,10 +1562,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -1542,10 +1573,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -1553,10 +1584,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -1564,10 +1595,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -1575,10 +1606,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -1586,10 +1617,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -1597,10 +1628,10 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C23" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -1608,10 +1639,10 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C24" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -1619,10 +1650,10 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>285</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -1630,10 +1661,10 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -1641,10 +1672,10 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -1652,10 +1683,10 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -1663,10 +1694,10 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -1674,10 +1705,10 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -1685,7 +1716,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C31" t="s">
         <v>3</v>
@@ -1696,10 +1727,10 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C32" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -1707,10 +1738,10 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C33" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -1718,10 +1749,10 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C34" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -1729,10 +1760,10 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -1740,10 +1771,10 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -1751,10 +1782,10 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>286</v>
       </c>
       <c r="C37" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -1762,10 +1793,10 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C38" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -1773,10 +1804,10 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C39" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -1784,10 +1815,10 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C40" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -1795,10 +1826,10 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>78</v>
+        <v>287</v>
       </c>
       <c r="C41" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -1806,10 +1837,10 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C42" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -1817,10 +1848,10 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C43" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -1828,10 +1859,10 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C44" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -1839,10 +1870,10 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C45" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -1850,10 +1881,10 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C46" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -1861,10 +1892,10 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C47" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -1872,10 +1903,10 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C48" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -1883,10 +1914,10 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C49" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -1894,10 +1925,10 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C50" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -1905,10 +1936,10 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>96</v>
+        <v>288</v>
       </c>
       <c r="C51" t="s">
-        <v>306</v>
+        <v>273</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -1916,10 +1947,10 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C52" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -1927,10 +1958,10 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C53" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -1938,10 +1969,10 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C54" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -1949,10 +1980,10 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C55" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -1960,10 +1991,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>104</v>
+        <v>289</v>
       </c>
       <c r="C56" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -1971,10 +2002,10 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>106</v>
+        <v>290</v>
       </c>
       <c r="C57" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -1982,10 +2013,10 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="C58" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -1993,10 +2024,10 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="C59" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
@@ -2004,10 +2035,10 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>112</v>
+        <v>291</v>
       </c>
       <c r="C60" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
@@ -2015,10 +2046,10 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C61" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
@@ -2026,10 +2057,10 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C62" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -2037,10 +2068,10 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C63" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -2048,10 +2079,10 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C64" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -2059,10 +2090,10 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C65" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -2070,10 +2101,10 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>123</v>
+        <v>314</v>
       </c>
       <c r="C66" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -2081,10 +2112,10 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>125</v>
+        <v>292</v>
       </c>
       <c r="C67" t="s">
-        <v>307</v>
+        <v>274</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
@@ -2092,10 +2123,10 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>126</v>
+        <v>293</v>
       </c>
       <c r="C68" t="s">
-        <v>307</v>
+        <v>274</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
@@ -2103,10 +2134,10 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C69" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
@@ -2114,10 +2145,10 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="C70" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
@@ -2125,10 +2156,10 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="C71" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -2136,10 +2167,10 @@
         <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>132</v>
+        <v>294</v>
       </c>
       <c r="C72" t="s">
-        <v>307</v>
+        <v>274</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -2147,13 +2178,13 @@
         <v>71</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>133</v>
+        <v>295</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>308</v>
+        <v>275</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>309</v>
+        <v>296</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
@@ -2161,10 +2192,10 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>134</v>
+        <v>297</v>
       </c>
       <c r="C74" t="s">
-        <v>307</v>
+        <v>274</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -2172,10 +2203,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="C75" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
@@ -2183,10 +2214,10 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="C76" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -2194,10 +2225,10 @@
         <v>75</v>
       </c>
       <c r="B77" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="C77" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
@@ -2205,10 +2236,10 @@
         <v>76</v>
       </c>
       <c r="B78" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="C78" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
@@ -2216,10 +2247,10 @@
         <v>77</v>
       </c>
       <c r="B79" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="C79" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -2227,7 +2258,7 @@
         <v>78</v>
       </c>
       <c r="B80" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="C80" t="s">
         <v>3</v>
@@ -2238,10 +2269,10 @@
         <v>79</v>
       </c>
       <c r="B81" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="C81" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -2249,7 +2280,7 @@
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>148</v>
+        <v>298</v>
       </c>
       <c r="C82" t="s">
         <v>3</v>
@@ -2260,7 +2291,7 @@
         <v>81</v>
       </c>
       <c r="B83" t="s">
-        <v>149</v>
+        <v>299</v>
       </c>
       <c r="C83" t="s">
         <v>3</v>
@@ -2271,7 +2302,7 @@
         <v>82</v>
       </c>
       <c r="B84" t="s">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="C84" t="s">
         <v>3</v>
@@ -2282,7 +2313,7 @@
         <v>83</v>
       </c>
       <c r="B85" t="s">
-        <v>151</v>
+        <v>301</v>
       </c>
       <c r="C85" t="s">
         <v>3</v>
@@ -2293,7 +2324,7 @@
         <v>84</v>
       </c>
       <c r="B86" t="s">
-        <v>152</v>
+        <v>302</v>
       </c>
       <c r="C86" t="s">
         <v>3</v>
@@ -2304,10 +2335,10 @@
         <v>85</v>
       </c>
       <c r="B87" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="C87" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -2315,10 +2346,10 @@
         <v>86</v>
       </c>
       <c r="B88" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="C88" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -2326,10 +2357,10 @@
         <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="C89" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -2337,10 +2368,10 @@
         <v>88</v>
       </c>
       <c r="B90" t="s">
-        <v>159</v>
+        <v>138</v>
       </c>
       <c r="C90" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -2348,10 +2379,10 @@
         <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>161</v>
+        <v>140</v>
       </c>
       <c r="C91" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -2359,7 +2390,7 @@
         <v>90</v>
       </c>
       <c r="B92" t="s">
-        <v>163</v>
+        <v>303</v>
       </c>
       <c r="C92" t="s">
         <v>3</v>
@@ -2370,10 +2401,10 @@
         <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>164</v>
+        <v>142</v>
       </c>
       <c r="C93" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -2381,10 +2412,10 @@
         <v>92</v>
       </c>
       <c r="B94" t="s">
-        <v>166</v>
+        <v>144</v>
       </c>
       <c r="C94" t="s">
-        <v>167</v>
+        <v>145</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -2392,10 +2423,10 @@
         <v>93</v>
       </c>
       <c r="B95" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
       <c r="C95" t="s">
-        <v>169</v>
+        <v>147</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -2403,10 +2434,10 @@
         <v>94</v>
       </c>
       <c r="B96" t="s">
-        <v>170</v>
+        <v>148</v>
       </c>
       <c r="C96" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -2414,10 +2445,10 @@
         <v>95</v>
       </c>
       <c r="B97" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="C97" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -2425,10 +2456,10 @@
         <v>96</v>
       </c>
       <c r="B98" t="s">
-        <v>174</v>
+        <v>152</v>
       </c>
       <c r="C98" t="s">
-        <v>175</v>
+        <v>153</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
@@ -2436,10 +2467,10 @@
         <v>97</v>
       </c>
       <c r="B99" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
       <c r="C99" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -2447,10 +2478,10 @@
         <v>98</v>
       </c>
       <c r="B100" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="C100" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -2458,10 +2489,10 @@
         <v>99</v>
       </c>
       <c r="B101" t="s">
-        <v>180</v>
+        <v>304</v>
       </c>
       <c r="C101" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -2469,10 +2500,10 @@
         <v>100</v>
       </c>
       <c r="B102" t="s">
-        <v>182</v>
+        <v>305</v>
       </c>
       <c r="C102" t="s">
-        <v>183</v>
+        <v>159</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -2480,7 +2511,7 @@
         <v>101</v>
       </c>
       <c r="B103" t="s">
-        <v>184</v>
+        <v>306</v>
       </c>
       <c r="C103" t="s">
         <v>3</v>
@@ -2491,7 +2522,7 @@
         <v>102</v>
       </c>
       <c r="B104" t="s">
-        <v>185</v>
+        <v>307</v>
       </c>
       <c r="C104" t="s">
         <v>3</v>
@@ -2502,10 +2533,10 @@
         <v>103</v>
       </c>
       <c r="B105" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="C105" t="s">
-        <v>187</v>
+        <v>161</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
@@ -2513,10 +2544,10 @@
         <v>104</v>
       </c>
       <c r="B106" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
       <c r="C106" t="s">
-        <v>189</v>
+        <v>163</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
@@ -2524,10 +2555,10 @@
         <v>105</v>
       </c>
       <c r="B107" t="s">
-        <v>190</v>
+        <v>164</v>
       </c>
       <c r="C107" t="s">
-        <v>191</v>
+        <v>165</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -2535,10 +2566,10 @@
         <v>106</v>
       </c>
       <c r="B108" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="C108" t="s">
-        <v>193</v>
+        <v>167</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
@@ -2546,10 +2577,10 @@
         <v>107</v>
       </c>
       <c r="B109" t="s">
-        <v>194</v>
+        <v>308</v>
       </c>
       <c r="C109" t="s">
-        <v>307</v>
+        <v>274</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -2557,7 +2588,7 @@
         <v>108</v>
       </c>
       <c r="B110" t="s">
-        <v>195</v>
+        <v>309</v>
       </c>
       <c r="C110" t="s">
         <v>3</v>
@@ -2568,10 +2599,10 @@
         <v>109</v>
       </c>
       <c r="B111" t="s">
-        <v>196</v>
+        <v>168</v>
       </c>
       <c r="C111" t="s">
-        <v>197</v>
+        <v>169</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -2579,10 +2610,10 @@
         <v>110</v>
       </c>
       <c r="B112" t="s">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="C112" t="s">
-        <v>199</v>
+        <v>171</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
@@ -2590,10 +2621,10 @@
         <v>111</v>
       </c>
       <c r="B113" t="s">
-        <v>200</v>
+        <v>172</v>
       </c>
       <c r="C113" t="s">
-        <v>201</v>
+        <v>173</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
@@ -2601,10 +2632,10 @@
         <v>112</v>
       </c>
       <c r="B114" t="s">
-        <v>202</v>
+        <v>174</v>
       </c>
       <c r="C114" t="s">
-        <v>203</v>
+        <v>175</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -2612,7 +2643,7 @@
         <v>113</v>
       </c>
       <c r="B115" t="s">
-        <v>204</v>
+        <v>310</v>
       </c>
       <c r="C115" t="s">
         <v>3</v>
@@ -2623,10 +2654,10 @@
         <v>114</v>
       </c>
       <c r="B116" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="C116" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
@@ -2634,10 +2665,10 @@
         <v>115</v>
       </c>
       <c r="B117" t="s">
-        <v>207</v>
+        <v>178</v>
       </c>
       <c r="C117" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -2645,10 +2676,10 @@
         <v>116</v>
       </c>
       <c r="B118" t="s">
-        <v>208</v>
+        <v>311</v>
       </c>
       <c r="C118" t="s">
-        <v>310</v>
+        <v>276</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -2656,10 +2687,10 @@
         <v>117</v>
       </c>
       <c r="B119" t="s">
-        <v>209</v>
+        <v>179</v>
       </c>
       <c r="C119" t="s">
-        <v>210</v>
+        <v>180</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
@@ -2667,10 +2698,10 @@
         <v>118</v>
       </c>
       <c r="B120" t="s">
-        <v>211</v>
+        <v>181</v>
       </c>
       <c r="C120" t="s">
-        <v>212</v>
+        <v>182</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
@@ -2678,10 +2709,10 @@
         <v>119</v>
       </c>
       <c r="B121" t="s">
-        <v>213</v>
+        <v>183</v>
       </c>
       <c r="C121" t="s">
-        <v>214</v>
+        <v>184</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
@@ -2689,10 +2720,10 @@
         <v>120</v>
       </c>
       <c r="B122" t="s">
-        <v>215</v>
+        <v>185</v>
       </c>
       <c r="C122" t="s">
-        <v>314</v>
+        <v>280</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -2700,10 +2731,10 @@
         <v>121</v>
       </c>
       <c r="B123" t="s">
-        <v>216</v>
+        <v>186</v>
       </c>
       <c r="C123" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -2711,10 +2742,10 @@
         <v>122</v>
       </c>
       <c r="B124" t="s">
-        <v>217</v>
+        <v>187</v>
       </c>
       <c r="C124" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -2722,10 +2753,10 @@
         <v>123</v>
       </c>
       <c r="B125" t="s">
-        <v>218</v>
+        <v>188</v>
       </c>
       <c r="C125" t="s">
-        <v>219</v>
+        <v>189</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -2733,10 +2764,10 @@
         <v>124</v>
       </c>
       <c r="B126" t="s">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C126" t="s">
-        <v>221</v>
+        <v>191</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -2744,10 +2775,10 @@
         <v>125</v>
       </c>
       <c r="B127" t="s">
-        <v>222</v>
+        <v>192</v>
       </c>
       <c r="C127" t="s">
-        <v>223</v>
+        <v>193</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
@@ -2755,10 +2786,10 @@
         <v>126</v>
       </c>
       <c r="B128" t="s">
-        <v>224</v>
+        <v>194</v>
       </c>
       <c r="C128" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
@@ -2766,10 +2797,10 @@
         <v>127</v>
       </c>
       <c r="B129" t="s">
-        <v>225</v>
+        <v>195</v>
       </c>
       <c r="C129" t="s">
-        <v>226</v>
+        <v>196</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
@@ -2777,10 +2808,10 @@
         <v>128</v>
       </c>
       <c r="B130" t="s">
-        <v>227</v>
+        <v>197</v>
       </c>
       <c r="C130" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
@@ -2788,10 +2819,10 @@
         <v>129</v>
       </c>
       <c r="B131" t="s">
-        <v>228</v>
+        <v>198</v>
       </c>
       <c r="C131" t="s">
-        <v>229</v>
+        <v>199</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
@@ -2799,10 +2830,10 @@
         <v>130</v>
       </c>
       <c r="B132" t="s">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="C132" t="s">
-        <v>231</v>
+        <v>201</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
@@ -2810,10 +2841,10 @@
         <v>131</v>
       </c>
       <c r="B133" t="s">
-        <v>232</v>
+        <v>202</v>
       </c>
       <c r="C133" t="s">
-        <v>233</v>
+        <v>203</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -2821,10 +2852,10 @@
         <v>132</v>
       </c>
       <c r="B134" t="s">
-        <v>234</v>
+        <v>204</v>
       </c>
       <c r="C134" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -2832,10 +2863,10 @@
         <v>133</v>
       </c>
       <c r="B135" t="s">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C135" t="s">
-        <v>236</v>
+        <v>206</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -2843,10 +2874,10 @@
         <v>134</v>
       </c>
       <c r="B136" t="s">
-        <v>237</v>
+        <v>207</v>
       </c>
       <c r="C136" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -2854,10 +2885,10 @@
         <v>135</v>
       </c>
       <c r="B137" t="s">
-        <v>238</v>
+        <v>208</v>
       </c>
       <c r="C137" t="s">
-        <v>239</v>
+        <v>209</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -2865,10 +2896,10 @@
         <v>136</v>
       </c>
       <c r="B138" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C138" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
@@ -2876,10 +2907,10 @@
         <v>137</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>242</v>
+        <v>312</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>311</v>
+        <v>277</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -2887,10 +2918,10 @@
         <v>138</v>
       </c>
       <c r="B140" t="s">
-        <v>243</v>
+        <v>212</v>
       </c>
       <c r="C140" t="s">
-        <v>244</v>
+        <v>213</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -2898,10 +2929,10 @@
         <v>139</v>
       </c>
       <c r="B141" t="s">
-        <v>245</v>
+        <v>214</v>
       </c>
       <c r="C141" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -2909,10 +2940,10 @@
         <v>140</v>
       </c>
       <c r="B142" t="s">
-        <v>246</v>
+        <v>215</v>
       </c>
       <c r="C142" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -2920,10 +2951,10 @@
         <v>141</v>
       </c>
       <c r="B143" t="s">
-        <v>247</v>
+        <v>216</v>
       </c>
       <c r="C143" t="s">
-        <v>248</v>
+        <v>217</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -2931,10 +2962,10 @@
         <v>142</v>
       </c>
       <c r="B144" t="s">
-        <v>249</v>
+        <v>218</v>
       </c>
       <c r="C144" t="s">
-        <v>250</v>
+        <v>219</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -2942,10 +2973,10 @@
         <v>143</v>
       </c>
       <c r="B145" t="s">
-        <v>251</v>
+        <v>313</v>
       </c>
       <c r="C145" t="s">
-        <v>252</v>
+        <v>220</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -2953,7 +2984,7 @@
         <v>144</v>
       </c>
       <c r="B146" t="s">
-        <v>253</v>
+        <v>221</v>
       </c>
       <c r="C146" t="s">
         <v>3</v>
@@ -2964,10 +2995,10 @@
         <v>145</v>
       </c>
       <c r="B147" t="s">
-        <v>254</v>
+        <v>222</v>
       </c>
       <c r="C147" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -2975,10 +3006,10 @@
         <v>146</v>
       </c>
       <c r="B148" t="s">
-        <v>255</v>
+        <v>223</v>
       </c>
       <c r="C148" t="s">
-        <v>256</v>
+        <v>224</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -2986,10 +3017,10 @@
         <v>147</v>
       </c>
       <c r="B149" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
       <c r="C149" t="s">
-        <v>258</v>
+        <v>226</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -2997,10 +3028,10 @@
         <v>148</v>
       </c>
       <c r="B150" t="s">
-        <v>259</v>
+        <v>227</v>
       </c>
       <c r="C150" t="s">
-        <v>260</v>
+        <v>228</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
@@ -3008,10 +3039,10 @@
         <v>149</v>
       </c>
       <c r="B151" t="s">
-        <v>261</v>
+        <v>229</v>
       </c>
       <c r="C151" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
@@ -3019,10 +3050,10 @@
         <v>150</v>
       </c>
       <c r="B152" t="s">
-        <v>262</v>
+        <v>230</v>
       </c>
       <c r="C152" t="s">
-        <v>263</v>
+        <v>231</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
@@ -3030,10 +3061,10 @@
         <v>151</v>
       </c>
       <c r="B153" t="s">
-        <v>264</v>
+        <v>232</v>
       </c>
       <c r="C153" t="s">
-        <v>265</v>
+        <v>233</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -3041,10 +3072,10 @@
         <v>152</v>
       </c>
       <c r="B154" t="s">
-        <v>266</v>
+        <v>234</v>
       </c>
       <c r="C154" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
@@ -3052,10 +3083,10 @@
         <v>153</v>
       </c>
       <c r="B155" t="s">
-        <v>267</v>
+        <v>235</v>
       </c>
       <c r="C155" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -3063,10 +3094,10 @@
         <v>154</v>
       </c>
       <c r="B156" t="s">
-        <v>268</v>
+        <v>236</v>
       </c>
       <c r="C156" t="s">
-        <v>269</v>
+        <v>237</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
@@ -3074,10 +3105,10 @@
         <v>155</v>
       </c>
       <c r="B157" t="s">
-        <v>270</v>
+        <v>238</v>
       </c>
       <c r="C157" t="s">
-        <v>271</v>
+        <v>239</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
@@ -3085,10 +3116,10 @@
         <v>156</v>
       </c>
       <c r="B158" t="s">
-        <v>272</v>
+        <v>240</v>
       </c>
       <c r="C158" t="s">
-        <v>273</v>
+        <v>241</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
@@ -3096,7 +3127,7 @@
         <v>157</v>
       </c>
       <c r="B159" t="s">
-        <v>274</v>
+        <v>242</v>
       </c>
       <c r="C159" t="s">
         <v>3</v>
@@ -3107,10 +3138,10 @@
         <v>158</v>
       </c>
       <c r="B160" t="s">
-        <v>275</v>
+        <v>243</v>
       </c>
       <c r="C160" t="s">
-        <v>276</v>
+        <v>244</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.2">
@@ -3118,7 +3149,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>277</v>
+        <v>245</v>
       </c>
       <c r="C161" s="3" t="s">
         <v>3</v>
@@ -3129,10 +3160,10 @@
         <v>160</v>
       </c>
       <c r="B162" t="s">
-        <v>278</v>
+        <v>246</v>
       </c>
       <c r="C162" t="s">
-        <v>279</v>
+        <v>247</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.2">
@@ -3140,10 +3171,10 @@
         <v>161</v>
       </c>
       <c r="B163" t="s">
-        <v>280</v>
+        <v>248</v>
       </c>
       <c r="C163" t="s">
-        <v>281</v>
+        <v>249</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.2">
@@ -3151,10 +3182,10 @@
         <v>162</v>
       </c>
       <c r="B164" t="s">
-        <v>282</v>
+        <v>250</v>
       </c>
       <c r="C164" t="s">
-        <v>283</v>
+        <v>251</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.2">
@@ -3162,10 +3193,10 @@
         <v>163</v>
       </c>
       <c r="B165" t="s">
-        <v>284</v>
+        <v>252</v>
       </c>
       <c r="C165" t="s">
-        <v>285</v>
+        <v>253</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.2">
@@ -3173,10 +3204,10 @@
         <v>164</v>
       </c>
       <c r="B166" t="s">
-        <v>286</v>
+        <v>254</v>
       </c>
       <c r="C166" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.2">
@@ -3184,10 +3215,10 @@
         <v>165</v>
       </c>
       <c r="B167" t="s">
-        <v>288</v>
+        <v>256</v>
       </c>
       <c r="C167" t="s">
-        <v>289</v>
+        <v>257</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.2">
@@ -3195,10 +3226,10 @@
         <v>166</v>
       </c>
       <c r="B168" t="s">
-        <v>290</v>
+        <v>258</v>
       </c>
       <c r="C168" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.2">
@@ -3206,10 +3237,10 @@
         <v>167</v>
       </c>
       <c r="B169" t="s">
-        <v>291</v>
+        <v>259</v>
       </c>
       <c r="C169" t="s">
-        <v>292</v>
+        <v>260</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.2">
@@ -3217,10 +3248,10 @@
         <v>168</v>
       </c>
       <c r="B170" t="s">
-        <v>293</v>
+        <v>261</v>
       </c>
       <c r="C170" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.2">
@@ -3228,13 +3259,13 @@
         <v>169</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>295</v>
+        <v>262</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>312</v>
+        <v>278</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>313</v>
+        <v>279</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.2">
@@ -3242,10 +3273,10 @@
         <v>170</v>
       </c>
       <c r="B172" t="s">
-        <v>296</v>
+        <v>263</v>
       </c>
       <c r="C172" t="s">
-        <v>297</v>
+        <v>264</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.2">
@@ -3253,10 +3284,10 @@
         <v>171</v>
       </c>
       <c r="B173" t="s">
-        <v>298</v>
+        <v>265</v>
       </c>
       <c r="C173" t="s">
-        <v>299</v>
+        <v>266</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.2">
@@ -3264,10 +3295,10 @@
         <v>172</v>
       </c>
       <c r="B174" t="s">
-        <v>300</v>
+        <v>267</v>
       </c>
       <c r="C174" t="s">
-        <v>305</v>
+        <v>272</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.2">
@@ -3275,10 +3306,10 @@
         <v>173</v>
       </c>
       <c r="B175" t="s">
-        <v>301</v>
+        <v>268</v>
       </c>
       <c r="C175" t="s">
-        <v>302</v>
+        <v>269</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.2">
@@ -3286,10 +3317,37 @@
         <v>174</v>
       </c>
       <c r="B176" t="s">
-        <v>303</v>
+        <v>270</v>
       </c>
       <c r="C176" t="s">
-        <v>304</v>
+        <v>271</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A177" s="4">
+        <v>175</v>
+      </c>
+      <c r="B177" t="s">
+        <v>316</v>
+      </c>
+      <c r="D177" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B178" t="s">
+        <v>317</v>
+      </c>
+      <c r="C178" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B179" t="s">
+        <v>319</v>
+      </c>
+      <c r="C179" t="s">
+        <v>320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>